<commit_message>
Make routine import tolerant to exercise name variants
</commit_message>
<xml_diff>
--- a/plantilla-rutina-gymos.xlsx
+++ b/plantilla-rutina-gymos.xlsx
@@ -461,7 +461,7 @@
         <v>Biblioteca</v>
       </c>
       <c r="B6" t="str">
-        <v>Selecciona ejercicios de Biblioteca: no inventes uno si allí existe una alternativa válida. Copia exactamente Ejercicio y _GymOS exercise en Rutina.</v>
+        <v>Selecciona ejercicios de Biblioteca: no inventes uno si allí existe una alternativa válida. Copia _GymOS exercise y Ejercicio cuando puedas.</v>
       </c>
     </row>
     <row r="7">
@@ -469,7 +469,7 @@
         <v>IDs</v>
       </c>
       <c r="B7" t="str">
-        <v>No traduzcas, abrevies ni modifiques IDs. Si el ejercicio no aparece en Biblioteca, deja _GymOS exercise vacío y conserva su nombre para el flujo existente.</v>
+        <v>_GymOS exercise es el identificador contractual: no lo traduzcas, abrevies, modifiques ni inventes. Ejercicio es descriptivo y GymOS puede normalizarlo automáticamente cuando el ID es válido.</v>
       </c>
     </row>
     <row r="8">
@@ -477,7 +477,7 @@
         <v>ChatGPT</v>
       </c>
       <c r="B8" t="str">
-        <v>Puede ayudarte a rellenar Sesiones y Rutina, pero debe respetar nombres, IDs, columnas y estructura de esta plantilla.</v>
+        <v>Puede ayudarte a rellenar Sesiones y Rutina. Debe copiar el ID y el nombre desde Biblioteca cuando pueda, respetando columnas y estructura.</v>
       </c>
     </row>
     <row r="9">

</xml_diff>